<commit_message>
Correlaciones: laminas regeneradas (2026-09-24)
</commit_message>
<xml_diff>
--- a/output/graficos_regionales_correlaciones/plot_nacional_correl_matriz_d_apoyopot_a_2019.xlsx
+++ b/output/graficos_regionales_correlaciones/plot_nacional_correl_matriz_d_apoyopot_a_2019.xlsx
@@ -111,7 +111,7 @@
     <t xml:space="preserve">Fecha de creación</t>
   </si>
   <si>
-    <t xml:space="preserve">2026-09-18 13:55</t>
+    <t xml:space="preserve">2026-09-24 00:46</t>
   </si>
   <si>
     <t xml:space="preserve">Fuente</t>
@@ -772,7 +772,7 @@
         <v>0.08</v>
       </c>
       <c r="D19" s="2" t="n">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="20">
@@ -786,7 +786,7 @@
         <v>0.13</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
     <row r="21">
@@ -800,7 +800,7 @@
         <v>-0.1</v>
       </c>
       <c r="D21" s="2" t="n">
-        <v>345</v>
+        <v>346</v>
       </c>
     </row>
   </sheetData>

</xml_diff>